<commit_message>
Actualizar preguntas de la encuesta según revisión del docente
- trabaja: se simplifica a Sí/No (antes 3 opciones); se ajustan las
  condicionales de donde_trabaja e ingresos para usar el nuevo valor
- area_sonido: pasa de opción múltiple a texto abierto (respuesta libre)
- entradas: se reformula en primera persona en vez de tercera
- 7 preguntas: ajuste de voseo a tuteo (tenés->tienes, vivís->vives, etc.)
- Tabla de preguntas (md + xlsx) regenerada con los cambios

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/encuesta/PREGUNTAS-tabla.xlsx
+++ b/encuesta/PREGUNTAS-tabla.xlsx
@@ -590,7 +590,7 @@
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>¿Qué edad tenés?</t>
+          <t>¿Qué edad tienes?</t>
         </is>
       </c>
       <c r="D2" s="3" t="inlineStr">
@@ -633,7 +633,7 @@
       </c>
       <c r="E3" s="4" t="inlineStr">
         <is>
-          <t>No, solo estudio / Sí, en algo de sonido / Sí, en otra área</t>
+          <t>No / Sí</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr"/>
@@ -845,7 +845,7 @@
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>¿Tenés otra profesión u oficio?</t>
+          <t>¿Tienes otra profesión u oficio?</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
@@ -919,7 +919,7 @@
       </c>
       <c r="C11" s="7" t="inlineStr">
         <is>
-          <t>¿Con quién vivís?</t>
+          <t>¿Con quién vives?</t>
         </is>
       </c>
       <c r="D11" s="6" t="inlineStr">
@@ -956,7 +956,7 @@
       </c>
       <c r="C12" s="7" t="inlineStr">
         <is>
-          <t>¿Ya tenés familia propia?</t>
+          <t>¿Ya tienes familia propia?</t>
         </is>
       </c>
       <c r="D12" s="6" t="inlineStr">
@@ -1137,7 +1137,7 @@
       </c>
       <c r="C17" s="10" t="inlineStr">
         <is>
-          <t>Cuando le pedís algo a una IA, ¿copiás y pegás o te detenés a leer?</t>
+          <t>Cuando le pides algo a una IA, ¿copias y pegas o te detienes a leer la respuesta?</t>
         </is>
       </c>
       <c r="D17" s="9" t="inlineStr">
@@ -1174,7 +1174,7 @@
       </c>
       <c r="C18" s="13" t="inlineStr">
         <is>
-          <t>¿Qué géneros musicales preferís?</t>
+          <t>¿Qué géneros musicales prefieres?</t>
         </is>
       </c>
       <c r="D18" s="12" t="inlineStr">
@@ -1211,7 +1211,7 @@
       </c>
       <c r="C19" s="13" t="inlineStr">
         <is>
-          <t>¿Sos músico?</t>
+          <t>¿Eres músico?</t>
         </is>
       </c>
       <c r="D19" s="12" t="inlineStr">
@@ -1421,7 +1421,7 @@
       </c>
       <c r="C25" s="13" t="inlineStr">
         <is>
-          <t>Hablando en general: entre estudiantes de sonido, ¿qué se estila más?</t>
+          <t>¿Al acudir a un concierto sueles pagar tu entrada?</t>
         </is>
       </c>
       <c r="D25" s="12" t="inlineStr">
@@ -1463,14 +1463,10 @@
       </c>
       <c r="D26" s="15" t="inlineStr">
         <is>
-          <t>Cerrada · opción múltiple</t>
-        </is>
-      </c>
-      <c r="E26" s="16" t="inlineStr">
-        <is>
-          <t>Acústica arquitectónica / Producción musical / Procesamiento de señales / Audio en vivo / Diseño sonoro / medios / Acústica ambiental y ruido / Audio inmersivo / espacial / Restauración y archivo</t>
-        </is>
-      </c>
+          <t>Abierta (texto libre)</t>
+        </is>
+      </c>
+      <c r="E26" s="16" t="inlineStr"/>
       <c r="F26" s="15" t="inlineStr"/>
       <c r="G26" s="14" t="inlineStr"/>
       <c r="H26" s="14" t="inlineStr">

</xml_diff>